<commit_message>
feat(beispiel): Muster Maschinenbau – full business year, company files, layout, messy documents
</commit_message>
<xml_diff>
--- a/plugin/beispiel-unordentlich/00_Eingang/ergebnis_2026-09.xlsx
+++ b/plugin/beispiel-unordentlich/00_Eingang/ergebnis_2026-09.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,17 +446,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Umsatz Service</t>
+          <t>Umsatz Ersatzteile</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>170.000,00</t>
+          <t>178.080,00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>101.139,00</t>
+          <t>154.249,59</t>
         </is>
       </c>
     </row>
@@ -468,17 +468,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Umsatz Ersatzteile</t>
+          <t>Umsatz Service</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>25.000,00</t>
+          <t>191.280,00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>111.380,21</t>
+          <t>219.719,20</t>
         </is>
       </c>
     </row>
@@ -490,17 +490,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Personalkosten</t>
+          <t>Umsatz Verträge</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>-61.000,00</t>
+          <t>66.000,00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-58.750,00</t>
+          <t>63.900,00</t>
         </is>
       </c>
     </row>
@@ -512,17 +512,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Material</t>
+          <t>Umsatz Schulung</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>-21.000,00</t>
+          <t>6.000,00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-24.310,00</t>
+          <t>10.150,00</t>
         </is>
       </c>
     </row>
@@ -534,17 +534,105 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Material</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-117.352,00</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-110.547,28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fremdleistung</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-14.000,00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-14.000,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Personalkosten</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>-153.600,00</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-143.750,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Gewährleistung</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>-4.000,00</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>-9.120,00</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>-6.000,00</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>-18.900,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Gemeinkostenumlage</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>-36.500,00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>-36.500,00</t>
         </is>
       </c>
     </row>

</xml_diff>